<commit_message>
Add unit tests for selective reshuffle functionality and create HR module
- Implemented unit tests in `tests/test_selective_reshuffle.py` to validate the selective reshuffle logic, ensuring that locked and unselected jobs are preserved.
- Added tests for rebuilding outputs from accepted sequences to maintain data integrity.
- Created an empty `HR/__init__.py` file to initialize the HR module.
</commit_message>
<xml_diff>
--- a/Flexar/BlueSG/rider_roster.xlsx
+++ b/Flexar/BlueSG/rider_roster.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -495,7 +495,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -793,12 +793,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Toa Payoh</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -811,53 +811,53 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Chong Zhen Yang (Michael)</t>
+          <t>Tee Boon Chuan (Jayson )</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Compassvale</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -868,25 +868,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mohammad Fareed Bin Mohammad Rashid</t>
+          <t>Chong Zhen Yang (Michael)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Queenstown</t>
+          <t>Compassvale</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -907,48 +907,48 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Syed Muhammad Faiq Bin Bagal</t>
+          <t>Abdul Rashid Bin Abdul Majid</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Marsiling</t>
+          <t>Balestier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Mohammad Fareed Bin Mohammad Rashid</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Queenstown</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -957,61 +957,86 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tee Boon Chuan (Jayson )</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Zhi Ming</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tampaines</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Lim Choon Yong Lester</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Bedok</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Normal</t>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1102,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1127,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1152,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1177,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1202,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1227,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1252,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1277,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1325,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Syed Muhammad Faiq Bin Bagal</t>
+          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Marsiling</t>
+          <t>Toa Payoh</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1314,173 +1339,173 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lim Choon Yong Lester</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bedok</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mohamed Sadhik Mohamed Yusof</t>
+          <t>Chong Zhen Yang (Michael)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orchard</t>
+          <t>Compassvale</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Safuwan</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tee Boon Chuan (Jayson )</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Zhi Ming</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Tee Boon Chuan (Jayson )</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mohammad Fareed Bin Mohammad Rashid</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Queens Town</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1489,11 +1514,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1584,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1609,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1634,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1659,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1684,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1709,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1734,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1759,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1825,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1850,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1875,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1900,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1925,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1950,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1975,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1975,7 +2000,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2066,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2091,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2116,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2141,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2166,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2191,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2216,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2241,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2266,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement WhatsApp request processor module with database and service layers
</commit_message>
<xml_diff>
--- a/Flexar/BlueSG/rider_roster.xlsx
+++ b/Flexar/BlueSG/rider_roster.xlsx
@@ -1774,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1832,42 +1832,42 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Aaron Singh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Chong Zhen Yang (Michael)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Compassvale</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -1882,21 +1882,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Safuwan</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1907,17 +1907,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aaron Singh</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1932,46 +1932,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Safuwan</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chong Zhen Yang (Michael)</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Compassvale</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1982,23 +1982,48 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mohammad Fareed Bin Mohammad Rashid</t>
+          <t>Arin Joshua Daniel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Queenstown</t>
+          <t>Ang Mo Kio</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mohamed Sadhik Mohamed Yusof</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>3</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2048,21 +2073,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lon</t>
+          <t>Ryan Oh</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Marsiling</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2073,21 +2098,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ryan Oh</t>
+          <t>Mohammad Fareed Bin Mohammad Rashid</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tampaines</t>
+          <t>Queenstown</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2098,12 +2123,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Aaron Singh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2112,7 +2137,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2123,21 +2148,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2148,17 +2173,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Toa Payoh</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -2166,19 +2191,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aaron Singh</t>
+          <t>Safuwan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2187,7 +2212,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2198,21 +2223,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Safuwan</t>
+          <t>Arin Joshua Daniel</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Ang Mo Kio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2223,12 +2248,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tee Boon Chuan (Jayson )</t>
+          <t>Lon</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Marsiling</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2237,7 +2262,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2248,25 +2273,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zhi Ming</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tampaines</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add comprehensive test suite for WhatsApp request processor and route planner
- Introduced unit tests for runtime support functions including repository path resolution, Python candidate order, HTTPS tunnel selection, atomic status write, and sensitive data redaction.
- Implemented tests for supervisor safety, ensuring environment variables are correctly set and supervisor processes are managed without conflicts.
- Added tests for WAAPI client to verify outbound gate functionality and default settings for rider and ops gates.
- Created batch scripts for starting and stopping the AMS WhatsApp Operations System.
- Developed extensive tests for the route planner, covering assignment validation, focus mode behavior, and route recalculation logic.
- Enhanced layout tests for Streamlit components in the route map viewer, ensuring proper dynamic behavior and styling.
</commit_message>
<xml_diff>
--- a/Flexar/BlueSG/rider_roster.xlsx
+++ b/Flexar/BlueSG/rider_roster.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,17 +452,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Mohammad Lutfi Dahnial Bin Radzaly</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Skengkang</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -477,17 +477,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aaron Singh</t>
+          <t>Chong Zhen Yang (Michael)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Compassvale</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -502,21 +502,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mohamed Sadhik Mohamed Yusof</t>
+          <t>Chean Zheng Tao Clifford</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Boon Keng</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -527,21 +527,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tee Boon Chuan (Jayson )</t>
+          <t>Asiah</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Skengkang</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -552,17 +552,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Syed Muhammad Faiq Bin Bagal</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Marsiling</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -577,21 +577,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Safuwan</t>
+          <t>Gary Koh Foo Choy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Skengkang</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -602,17 +602,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
+          <t>Abdul Rashid Bin Abdul Majid</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Toa Payoh</t>
+          <t>Balestier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -627,17 +627,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zhi Ming</t>
+          <t>Arin Joshua Daniel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tampaines</t>
+          <t>Geylang</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -652,37 +652,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chong Zhen Yang (Michael)</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Compassvale</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Zhi Ming</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -702,50 +702,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mohammad Fareed Bin Mohammad Rashid</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Queenstown</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add tests, UI components, and SSRS integration for report generation and management
- Introduced new test fixtures for SSRS catalog responses and folder pages.
- Implemented tests for incremental parsing, RDL parsing, and SQL safety.
- Developed UI components for downloading reports and managing SQL queries.
- Added functionality to handle ZIP archives and RDL files in the report tool.
- Enhanced SSRS client to normalize catalog items and validate report content.
- Created a structured approach for managing crawl states and download jobs.
- Ensured safety checks for SQL queries to prevent unsafe operations.
</commit_message>
<xml_diff>
--- a/Flexar/BlueSG/rider_roster.xlsx
+++ b/Flexar/BlueSG/rider_roster.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,17 +768,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sadiq Batcha Mohamed Yusoof Mahadir</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Toa Payoh</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -786,24 +786,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -811,14 +811,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tee Boon Chuan (Jayson )</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -843,21 +843,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chong Zhen Yang (Michael)</t>
+          <t>Abdul Rashid Bin Abdul Majid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Compassvale</t>
+          <t>Balestier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -868,12 +868,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Safuwan</t>
+          <t>Syed Muhammad Faiq Bin Bagal</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Marsiling</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -893,12 +893,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Mohammad Fareed Bin Mohammad Rashid</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Queenstown</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -918,21 +918,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mohammad Fareed Bin Mohammad Rashid</t>
+          <t>Asiah</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Queenstown</t>
+          <t>Skengkang</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -943,21 +943,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Hidayat</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -968,21 +968,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zhi Ming</t>
+          <t>Jasmet Singh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tampaines</t>
+          <t>Skengkang</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -993,12 +993,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lim Choon Yong Lester</t>
+          <t>Samuel Kasi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bedok</t>
+          <t>Yew Tee</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1007,11 +1007,111 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Chean Zheng Tao Clifford</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tampaines</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gary Koh Foo Choy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skengkang</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Arin Joshua Daniel</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ang Mo Kio</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mohamed Sadhik Mohamed Yusof</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add unit tests for vehicle route optimizer functionality
- Implement tests to verify the fixed terminal display for live activity.
- Ensure assignment progress events correctly include car and final rider details.
- Utilize monkeypatching to simulate travel cost retrieval during optimization.
</commit_message>
<xml_diff>
--- a/Flexar/BlueSG/rider_roster.xlsx
+++ b/Flexar/BlueSG/rider_roster.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,12 +452,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mohammad Lutfi Dahnial Bin Radzaly</t>
+          <t>Arin Joshua Daniel</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Skengkang</t>
+          <t>Ang Mo Kio</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -477,17 +477,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chong Zhen Yang (Michael)</t>
+          <t>Ooi Kin Soon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Compassvale</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -502,7 +502,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Chean Zheng Tao Clifford</t>
+          <t>Matthias Laurence</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -527,21 +527,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Asiah</t>
+          <t>Syed Muhammad Faiq Bin Bagal</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Skengkang</t>
+          <t>Marsiling</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -552,21 +552,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ooi Kin Soon</t>
+          <t>Chong Zhen Yang (Michael)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Compassvale</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North-East</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -602,21 +602,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abdul Rashid Bin Abdul Majid</t>
+          <t>Safuwan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Balestier</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -627,37 +627,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arin Joshua Daniel</t>
+          <t>Lim Choon Yong Lester</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Geylang</t>
+          <t>Bedok</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>North-East</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chen Yen Zong (El-Tian)</t>
+          <t>Zhi Ming</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Whampoa</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -677,12 +677,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zhi Ming</t>
+          <t>Chen Yen Zong (El-Tian)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tampaines</t>
+          <t>Whampoa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lim Choon Yong Lester</t>
+          <t>Chean Zheng Tao Clifford</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bedok</t>
+          <t>Tampaines</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -716,11 +716,36 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Vincent</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tampaines</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>

</xml_diff>